<commit_message>
docs(ld): question drafts updated with HR confirmations (Sick Leave: Manager and above; travel claims: 7 days)
Policy draft: the two amber checks are now recorded as confirmed. First bank draft: the 30-day travel/expense claim
question is removed (92 questions) and the Sick Leave question names its eligibility.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/LD_Policy_Questions_DRAFT.xlsx
+++ b/docs/LD_Policy_Questions_DRAFT.xlsx
@@ -5892,11 +5892,7 @@
           <t>Attendance &amp; Leave Policy (P002) · Leave Entitlement / Sick Leave</t>
         </is>
       </c>
-      <c r="H33" s="5" t="inlineStr">
-        <is>
-          <t>Confirm this is really intended: the earlier draft question bank (from the training guide) assumes Sick Leave for all.</t>
-        </is>
-      </c>
+      <c r="H33" s="2" t="inlineStr"/>
       <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="inlineStr"/>
       <c r="K33" s="2" t="inlineStr"/>
@@ -6923,11 +6919,7 @@
           <t>Travel Policy (P008, wef 1 Jul 2026) · Travel Advance</t>
         </is>
       </c>
-      <c r="H62" s="5" t="inlineStr">
-        <is>
-          <t>The training guide says expense claims must be submitted within 30 days through Maxvolt One. Confirm which rule applies to travel claims before using this question.</t>
-        </is>
-      </c>
+      <c r="H62" s="2" t="inlineStr"/>
       <c r="I62" s="2" t="inlineStr"/>
       <c r="J62" s="2" t="inlineStr"/>
       <c r="K62" s="2" t="inlineStr"/>
@@ -7937,7 +7929,7 @@
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>• Travel claims: the Travel Policy says the expense statement is due within 7 business days of resuming work; the training guide says expense claims are due within 30 days. One of them needs to change, or the two need to be explained as different claim types.</t>
+          <t>• CONFIRMED by HR on 26 Oct 2026: travel claims (Travel Expense Statement) are due within 7 business days of resuming work. The training guide and the induction step G03-5 still say expense claims are due within 30 days — correct the wording to match (the older question on the 30-day rule has been removed from the first question-bank draft).</t>
         </is>
       </c>
     </row>
@@ -7951,7 +7943,7 @@
     <row r="27" ht="32" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>• Attendance &amp; Leave: Sick Leave is stated as applicable only to Manager level and above. If that is intended, the earlier question-bank draft (which assumed Sick Leave for everyone) needs that row corrected.</t>
+          <t>• CONFIRMED by HR on 26 Oct 2026: Sick Leave is granted only to Manager level and above (the question on it says so).</t>
         </is>
       </c>
     </row>

</xml_diff>